<commit_message>
Wedding Venue EN revisión D174: entregables remontados, gates verdes, REVISION-FINAL y ERRATAS-ES
2 B · 5 M · 21 m. Tras la ronda: D15 VERDE, G1-G9 VERDE, barrido 0, censo 0, regresión 30/30 y 2.ª pasada con sha
canónico igual en los 5; Word en 25 páginas y contrato en 12. La calculadora no cambia.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/wedding-venue-business-plan/wedding-venue-financial-projections.xlsx
+++ b/astro-site/public/dl/wedding-venue-business-plan/wedding-venue-financial-projections.xlsx
@@ -825,7 +825,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Menu price incl. sales tax (calculated)</t>
+          <t>Revenue per guest incl. sales tax (calculated)</t>
         </is>
       </c>
       <c r="B9" s="80">
@@ -1236,7 +1236,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Sales tax rate on sales</t>
+          <t>Sales tax rate on food sales (not used: the venue sells no food)</t>
         </is>
       </c>
       <c r="B39" s="63" t="n">
@@ -1251,7 +1251,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sales tax rate on alcohol to go</t>
+          <t>General sales tax rate (reference only: the rates used are on the P&amp;L)</t>
         </is>
       </c>
       <c r="B40" s="63" t="n">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>General example rate, 8%. In this plan it applies to everything the venue bills as rental and services; the caterer commission is taxed at 0% in the model, and the venue's purchases carry no recoverable credit. The venue does not sell food or beverage: the caterer bills the menu and the bar. Some states do not tax venue fees at all: confirm yours with your state department of revenue</t>
+          <t>REFERENCE ONLY: no formula reads this cell. The sales tax the venue collects is typed in the "Sales tax rate on the line (%)" column of the "3-Year P&amp;L": 8% on venue rental &amp; services (G10) and 0% on the caterer commission (G11) in the example. The venue does not sell food or beverage: the caterer bills the menu and the bar. Some states do not tax venue fees at all: confirm yours with your state department of revenue</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="D10" s="28" t="inlineStr">
         <is>
-          <t>Sprinklers need city water; a tank and fire pump, a new septic system or a strict county can double this line. Whether you need them depends on the fire code your county has adopted: ask the building official and the fire marshal in writing, and get local quotes</t>
+          <t>Sprinklers need enough water flow: without city water, a tank and fire pump, a new septic system or a strict county can double this line. Whether you need them depends on the fire code your county has adopted: ask the building official and the fire marshal in writing, and get local quotes</t>
         </is>
       </c>
       <c r="E10" s="31" t="inlineStr">
@@ -6139,7 +6139,7 @@
         </is>
       </c>
       <c r="B20" s="78" t="n">
-        <v>9.199999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C20" s="28" t="n"/>
       <c r="D20" s="28" t="n"/>
@@ -6161,7 +6161,7 @@
         </is>
       </c>
       <c r="B21" s="78" t="n">
-        <v>2.3</v>
+        <v>2.35</v>
       </c>
       <c r="C21" s="28" t="n"/>
       <c r="D21" s="28" t="n"/>
@@ -6228,7 +6228,7 @@
       </c>
       <c r="B24" s="39">
         <f>IFERROR(IF(OR(B20="",B21="",'0. Assumptions'!$B$6=""),"",B20*B21*'0. Assumptions'!$B$6+B22*B23*'0. Assumptions'!$B$6),"")</f>
-        <v>5716.0</v>
+        <v>5879.5</v>
       </c>
       <c r="C24" s="28" t="n"/>
       <c r="D24" s="28" t="n"/>
@@ -6266,7 +6266,7 @@
       </c>
       <c r="B26" s="66">
         <f>IFERROR(B25/B24,"")</f>
-        <v>1.1910426871938418</v>
+        <v>1.1579215919721064</v>
       </c>
       <c r="C26" s="28" t="n"/>
       <c r="D26" s="28" t="n"/>
@@ -6871,7 +6871,7 @@
       </c>
       <c r="D36" s="46" t="inlineStr">
         <is>
-          <t>Weddings 130 guests × ($9,000 site fee + 10% of $110 F&amp;B per guest), corporate 70 × ($3,500 + 10% of $50), private 80 × ($4,000 + 10% of $55), micro 30 × ($2,000 + 10% of $80), excl. sales tax</t>
+          <t>Per event, excl. sales tax: wedding (130 guests) $9,000 site fee + 10% of $110 F&amp;B per guest; corporate (70) $3,500 + 10% of $50; private (80) $4,000 + 10% of $55; micro wedding (30) $2,000 + 10% of $80</t>
         </is>
       </c>
       <c r="E36" s="28" t="n"/>
@@ -7114,17 +7114,17 @@
       </c>
       <c r="B47" s="28" t="inlineStr">
         <is>
-          <t>A well that serves your guests may count as a public water system</t>
+          <t>A public water system if it regularly serves an average of 25 or more people a day at least 60 days a year</t>
         </is>
       </c>
       <c r="C47" s="28" t="inlineStr">
         <is>
-          <t>Ask your state drinking water program</t>
+          <t>40 CFR 141.2 (EPA); your state drinking water program applies it</t>
         </is>
       </c>
       <c r="D47" s="46" t="inlineStr">
         <is>
-          <t>Testing and a permit before the first event</t>
+          <t>Ask your state program about testing and a permit before the first event</t>
         </is>
       </c>
       <c r="E47" s="28" t="n"/>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="O20" s="28" t="inlineStr">
         <is>
-          <t>Cash only leaves when the quarter's result is positive. Months without a settlement are left blank, not zero. The cell turns RED when the payment takes more cash than is left that month. The model settles quarterly, in the month after each plan quarter (Months 4, 7 and 10: December, March and June with Month 1 in September; the fourth quarter is remitted in Month 13): if your state requires monthly filing, expect smaller payments every month instead</t>
+          <t>Cash only leaves when the quarter's result is positive. Months without a settlement are left blank, not zero. The cell turns RED when the payment takes more cash than is left that month. The model settles quarterly, in the month after each plan quarter (Months 4, 7 and 10: June, September and December with Month 1 in March; the fourth quarter is remitted in Month 13): if your state requires monthly filing, expect smaller payments every month instead</t>
         </is>
       </c>
     </row>

</xml_diff>